<commit_message>
Note that all scores are pre-use reference scores; add review memo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019DmDj1ymZTw123to8fqhuT
</commit_message>
<xml_diff>
--- a/catalog/list_01_英語圏_前半_採点.xlsx
+++ b/catalog/list_01_英語圏_前半_採点.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,11 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -124,6 +129,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -43910,7 +43918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44101,7 +44109,17 @@
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="8" t="n"/>
     </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>・【重要】点数はすべて「使う前に、説明文など外から見て付けた参考点数」です。アイデア・機能の見込みを示すもので、動作の速さ・使いやすさ（手数の少なさ）・堅牢さ（安定性）などの実装品質は含みません。点差の小さいものの優劣は判断せず、傾向を見る目安として使ってください。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>